<commit_message>
11:52 with 302+ images
</commit_message>
<xml_diff>
--- a/神社檔案/temple2.xlsx
+++ b/神社檔案/temple2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaish_mac/Desktop/DRHS/for github/mapu2/神社檔案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93D82CCE-B091-6045-9685-B5B1661BCFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF77945-F0A2-6348-AAAD-AFF7633C1C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>編號</t>
   </si>
@@ -731,13 +731,290 @@
   </si>
   <si>
     <t>東勢神社於1937年落成，1945年升格為鄉社，位於東勢市區附近山丘，景觀視野良好。戰後原址設立東勢工業技術講習班，後發展為東勢高工。雖校舍已遷移，舊校區仍保留參道與狛犬等神社遺跡。</t>
+  </si>
+  <si>
+    <t>開山神社</t>
+  </si>
+  <si>
+    <t>延平郡王祠</t>
+  </si>
+  <si>
+    <t>花蓮港神社</t>
+  </si>
+  <si>
+    <t>花蓮縣忠烈祠</t>
+  </si>
+  <si>
+    <t>台東神社</t>
+  </si>
+  <si>
+    <t>台東縣忠烈祠</t>
+  </si>
+  <si>
+    <t>阿緱神社</t>
+  </si>
+  <si>
+    <t>屏東忠烈祠</t>
+  </si>
+  <si>
+    <t>宜蘭神社</t>
+  </si>
+  <si>
+    <t>宜蘭忠烈祠</t>
+  </si>
+  <si>
+    <t>高雄神社</t>
+  </si>
+  <si>
+    <t>高雄忠烈祠</t>
+  </si>
+  <si>
+    <t>基隆神社</t>
+  </si>
+  <si>
+    <t>主普壇周邊</t>
+  </si>
+  <si>
+    <t>澎湖神社</t>
+  </si>
+  <si>
+    <t>澎湖忠烈祠</t>
+  </si>
+  <si>
+    <t>苗栗神社</t>
+  </si>
+  <si>
+    <t>苗栗縣忠烈祠</t>
+  </si>
+  <si>
+    <t>桃園神社</t>
+  </si>
+  <si>
+    <t>桃園忠烈祠暨神社文化園區</t>
+  </si>
+  <si>
+    <t>北港神社</t>
+  </si>
+  <si>
+    <t>北港朝天宮周邊遺址</t>
+  </si>
+  <si>
+    <r>
+      <t>臺南市中西區開山路</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>152</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>號</t>
+    </r>
+  </si>
+  <si>
+    <t>由開山王廟改設神社，祭祀鄭成功。</t>
+  </si>
+  <si>
+    <r>
+      <t>花蓮縣花蓮市復興新村</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>82</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>號（美崙山）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>原於</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>1916</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年鎮座，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>1921</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年列格縣社。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>臺東縣臺東市博愛路</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>425</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>號附近</t>
+    </r>
+  </si>
+  <si>
+    <t>位於鯉魚山，為臺東廳主要神社。</t>
+  </si>
+  <si>
+    <t>屏東縣屏東市公園路</t>
+  </si>
+  <si>
+    <t>阿緱為屏東舊稱，神社位於現中山公園一帶。</t>
+  </si>
+  <si>
+    <t>宜蘭縣宜蘭市復興路三段</t>
+  </si>
+  <si>
+    <t>現存鳥居、參道及部分遺構。</t>
+  </si>
+  <si>
+    <r>
+      <t>高雄市鼓山區忠義路</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>號</t>
+    </r>
+  </si>
+  <si>
+    <t>位於壽山山麓，戰後改為忠烈祠。</t>
+  </si>
+  <si>
+    <t>基隆市中正區壽山路</t>
+  </si>
+  <si>
+    <t>位於基隆市壽山，現遺跡有限。</t>
+  </si>
+  <si>
+    <t>澎湖縣馬公市介壽路</t>
+  </si>
+  <si>
+    <t>澎湖廳主要神社，位於金龍頭地區。</t>
+  </si>
+  <si>
+    <t>苗栗縣苗栗市建功里自治路</t>
+  </si>
+  <si>
+    <t>戰爭末期升格設立，存續時間極短。</t>
+  </si>
+  <si>
+    <r>
+      <t>桃園市桃園區成功路三段</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="PingFang TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>號</t>
+    </r>
+  </si>
+  <si>
+    <t>現存臺灣保存最完整的神社建築群。</t>
+  </si>
+  <si>
+    <t>雲林縣北港鎮北港街區</t>
+  </si>
+  <si>
+    <t>日治末期設立，戰後迅速廢止。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -819,6 +1096,19 @@
       <family val="4"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="PingFang TC"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -840,7 +1130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -859,6 +1149,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1161,7 +1453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12.3984375" customWidth="1"/>
@@ -1898,6 +2190,325 @@
         <v>104</v>
       </c>
     </row>
+    <row r="26" spans="1:9" ht="16">
+      <c r="A26" s="12">
+        <v>302</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E26" s="12">
+        <v>22.9909</v>
+      </c>
+      <c r="F26" s="12">
+        <v>120.2043</v>
+      </c>
+      <c r="G26" s="12">
+        <v>1897</v>
+      </c>
+      <c r="H26" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="16">
+      <c r="A27" s="12">
+        <v>303</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E27" s="12">
+        <v>23.985099999999999</v>
+      </c>
+      <c r="F27" s="12">
+        <v>121.6108</v>
+      </c>
+      <c r="G27" s="12">
+        <v>1921</v>
+      </c>
+      <c r="H27" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="16">
+      <c r="A28" s="12">
+        <v>304</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="E28" s="12">
+        <v>22.758500000000002</v>
+      </c>
+      <c r="F28" s="12">
+        <v>121.1444</v>
+      </c>
+      <c r="G28" s="12">
+        <v>1924</v>
+      </c>
+      <c r="H28" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="16">
+      <c r="A29" s="12">
+        <v>305</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E29" s="12">
+        <v>22.6737</v>
+      </c>
+      <c r="F29" s="12">
+        <v>120.48860000000001</v>
+      </c>
+      <c r="G29" s="12">
+        <v>1926</v>
+      </c>
+      <c r="H29" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="16">
+      <c r="A30" s="12">
+        <v>306</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E30" s="12">
+        <v>24.7578</v>
+      </c>
+      <c r="F30" s="12">
+        <v>121.7533</v>
+      </c>
+      <c r="G30" s="12">
+        <v>1927</v>
+      </c>
+      <c r="H30" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="16">
+      <c r="A31" s="12">
+        <v>307</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31" s="12">
+        <v>22.637499999999999</v>
+      </c>
+      <c r="F31" s="12">
+        <v>120.27549999999999</v>
+      </c>
+      <c r="G31" s="12">
+        <v>1932</v>
+      </c>
+      <c r="H31" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="16">
+      <c r="A32" s="12">
+        <v>308</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" s="12">
+        <v>25.130299999999998</v>
+      </c>
+      <c r="F32" s="12">
+        <v>121.7448</v>
+      </c>
+      <c r="G32" s="12">
+        <v>1936</v>
+      </c>
+      <c r="H32" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I32" s="13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="16">
+      <c r="A33" s="12">
+        <v>309</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E33" s="12">
+        <v>23.5654</v>
+      </c>
+      <c r="F33" s="12">
+        <v>119.5675</v>
+      </c>
+      <c r="G33" s="12">
+        <v>1938</v>
+      </c>
+      <c r="H33" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I33" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="16">
+      <c r="A34" s="12">
+        <v>310</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="E34" s="12">
+        <v>24.564800000000002</v>
+      </c>
+      <c r="F34" s="12">
+        <v>120.82040000000001</v>
+      </c>
+      <c r="G34" s="12">
+        <v>1945</v>
+      </c>
+      <c r="H34" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I34" s="13" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="16">
+      <c r="A35" s="12">
+        <v>311</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" s="12">
+        <v>24.9985</v>
+      </c>
+      <c r="F35" s="12">
+        <v>121.3249</v>
+      </c>
+      <c r="G35" s="12">
+        <v>1945</v>
+      </c>
+      <c r="H35" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I35" s="13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="16">
+      <c r="A36" s="12">
+        <v>312</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E36" s="12">
+        <v>23.575800000000001</v>
+      </c>
+      <c r="F36" s="12">
+        <v>120.3044</v>
+      </c>
+      <c r="G36" s="12">
+        <v>1945</v>
+      </c>
+      <c r="H36" s="12">
+        <v>1945</v>
+      </c>
+      <c r="I36" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>